<commit_message>
Atualiza arquivos Excel de registro
</commit_message>
<xml_diff>
--- a/estado/registroRegional.xlsx
+++ b/estado/registroRegional.xlsx
@@ -7939,7 +7939,7 @@
         <v>69312</v>
       </c>
       <c r="K92" t="n">
-        <v>456</v>
+        <v>464</v>
       </c>
     </row>
     <row r="93">
@@ -11414,7 +11414,7 @@
         <v>79221</v>
       </c>
       <c r="K92" t="n">
-        <v>622</v>
+        <v>631</v>
       </c>
     </row>
     <row r="93">
@@ -14902,7 +14902,7 @@
         <v>140427</v>
       </c>
       <c r="K92" t="n">
-        <v>38</v>
+        <v>145</v>
       </c>
     </row>
     <row r="93">
@@ -18377,7 +18377,7 @@
         <v>79201</v>
       </c>
       <c r="K92" t="n">
-        <v>384</v>
+        <v>391</v>
       </c>
     </row>
     <row r="93">
@@ -21834,7 +21834,7 @@
         <v>0.0003700876867500918</v>
       </c>
       <c r="E92" t="n">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="F92" t="n">
         <v>1842767</v>
@@ -21852,7 +21852,7 @@
         <v>189345</v>
       </c>
       <c r="K92" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="93">
@@ -25327,7 +25327,7 @@
         <v>61273</v>
       </c>
       <c r="K92" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
     </row>
     <row r="93">
@@ -28802,7 +28802,7 @@
         <v>66065</v>
       </c>
       <c r="K92" t="n">
-        <v>272</v>
+        <v>290</v>
       </c>
     </row>
     <row r="93">
@@ -32277,7 +32277,7 @@
         <v>54759</v>
       </c>
       <c r="K92" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="93">
@@ -35752,7 +35752,7 @@
         <v>56306</v>
       </c>
       <c r="K92" t="n">
-        <v>158</v>
+        <v>170</v>
       </c>
     </row>
     <row r="93">
@@ -39227,7 +39227,7 @@
         <v>52792</v>
       </c>
       <c r="K92" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="93">

</xml_diff>